<commit_message>
daily order build 2026-06-16
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-06-17
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -453,13 +453,13 @@
         <v>385</v>
       </c>
       <c r="C2" t="n">
-        <v>440147</v>
+        <v>440099</v>
       </c>
       <c r="D2" t="n">
-        <v>257139</v>
+        <v>257799</v>
       </c>
       <c r="E2" t="n">
-        <v>181590</v>
+        <v>180952</v>
       </c>
     </row>
     <row r="3">
@@ -475,10 +475,10 @@
         <v>23230</v>
       </c>
       <c r="D3" t="n">
-        <v>8024</v>
+        <v>7895</v>
       </c>
       <c r="E3" t="n">
-        <v>15034</v>
+        <v>15140</v>
       </c>
     </row>
     <row r="4">
@@ -491,13 +491,13 @@
         <v>866</v>
       </c>
       <c r="C4" t="n">
-        <v>325004</v>
+        <v>322393</v>
       </c>
       <c r="D4" t="n">
-        <v>111758</v>
+        <v>110759</v>
       </c>
       <c r="E4" t="n">
-        <v>203247</v>
+        <v>201146</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="C5" t="n">
-        <v>575484</v>
+        <v>576018</v>
       </c>
       <c r="D5" t="n">
-        <v>212171</v>
+        <v>210051</v>
       </c>
       <c r="E5" t="n">
-        <v>349440</v>
+        <v>351887</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C6" t="n">
-        <v>46516</v>
+        <v>46537</v>
       </c>
       <c r="D6" t="n">
-        <v>22755</v>
+        <v>22830</v>
       </c>
       <c r="E6" t="n">
-        <v>22259</v>
+        <v>22211</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-06-18
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -453,13 +453,13 @@
         <v>321</v>
       </c>
       <c r="C2" t="n">
-        <v>440099</v>
+        <v>440135</v>
       </c>
       <c r="D2" t="n">
-        <v>257799</v>
+        <v>257216</v>
       </c>
       <c r="E2" t="n">
-        <v>151733</v>
+        <v>152195</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C3" t="n">
-        <v>23230</v>
+        <v>23159</v>
       </c>
       <c r="D3" t="n">
-        <v>7895</v>
+        <v>7915</v>
       </c>
       <c r="E3" t="n">
-        <v>11612</v>
+        <v>11097</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>648</v>
+        <v>645</v>
       </c>
       <c r="C4" t="n">
-        <v>322393</v>
+        <v>323496</v>
       </c>
       <c r="D4" t="n">
-        <v>110759</v>
+        <v>111933</v>
       </c>
       <c r="E4" t="n">
-        <v>152472</v>
+        <v>136943</v>
       </c>
     </row>
     <row r="5">
@@ -510,13 +510,13 @@
         <v>502</v>
       </c>
       <c r="C5" t="n">
-        <v>576018</v>
+        <v>575785</v>
       </c>
       <c r="D5" t="n">
-        <v>210051</v>
+        <v>211830</v>
       </c>
       <c r="E5" t="n">
-        <v>214834</v>
+        <v>213976</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C6" t="n">
-        <v>46537</v>
+        <v>46458</v>
       </c>
       <c r="D6" t="n">
-        <v>22830</v>
+        <v>22620</v>
       </c>
       <c r="E6" t="n">
-        <v>21173</v>
+        <v>21360</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-06-19
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C2" t="n">
-        <v>440135</v>
+        <v>440111</v>
       </c>
       <c r="D2" t="n">
-        <v>257216</v>
+        <v>256224</v>
       </c>
       <c r="E2" t="n">
-        <v>152195</v>
+        <v>154115</v>
       </c>
     </row>
     <row r="3">
@@ -472,13 +472,13 @@
         <v>54</v>
       </c>
       <c r="C3" t="n">
-        <v>23159</v>
+        <v>23160</v>
       </c>
       <c r="D3" t="n">
-        <v>7915</v>
+        <v>7978</v>
       </c>
       <c r="E3" t="n">
-        <v>11097</v>
+        <v>11081</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="C4" t="n">
-        <v>323496</v>
+        <v>321849</v>
       </c>
       <c r="D4" t="n">
-        <v>111933</v>
+        <v>111979</v>
       </c>
       <c r="E4" t="n">
-        <v>136943</v>
+        <v>135982</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="C5" t="n">
-        <v>575785</v>
+        <v>578089</v>
       </c>
       <c r="D5" t="n">
-        <v>211830</v>
+        <v>212509</v>
       </c>
       <c r="E5" t="n">
-        <v>213976</v>
+        <v>213224</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C6" t="n">
-        <v>46458</v>
+        <v>46501</v>
       </c>
       <c r="D6" t="n">
-        <v>22620</v>
+        <v>22546</v>
       </c>
       <c r="E6" t="n">
-        <v>21360</v>
+        <v>21588</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-06-20
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C2" t="n">
-        <v>440111</v>
+        <v>440210</v>
       </c>
       <c r="D2" t="n">
-        <v>256224</v>
+        <v>255695</v>
       </c>
       <c r="E2" t="n">
-        <v>154115</v>
+        <v>154996</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C3" t="n">
-        <v>23160</v>
+        <v>23105</v>
       </c>
       <c r="D3" t="n">
-        <v>7978</v>
+        <v>7274</v>
       </c>
       <c r="E3" t="n">
-        <v>11081</v>
+        <v>11429</v>
       </c>
     </row>
     <row r="4">
@@ -491,13 +491,13 @@
         <v>648</v>
       </c>
       <c r="C4" t="n">
-        <v>321849</v>
+        <v>324166</v>
       </c>
       <c r="D4" t="n">
-        <v>111979</v>
+        <v>111542</v>
       </c>
       <c r="E4" t="n">
-        <v>135982</v>
+        <v>137877</v>
       </c>
     </row>
     <row r="5">
@@ -510,13 +510,13 @@
         <v>500</v>
       </c>
       <c r="C5" t="n">
-        <v>578089</v>
+        <v>578114</v>
       </c>
       <c r="D5" t="n">
-        <v>212509</v>
+        <v>207662</v>
       </c>
       <c r="E5" t="n">
-        <v>213224</v>
+        <v>215232</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C6" t="n">
-        <v>46501</v>
+        <v>46509</v>
       </c>
       <c r="D6" t="n">
-        <v>22546</v>
+        <v>22292</v>
       </c>
       <c r="E6" t="n">
-        <v>21588</v>
+        <v>21725</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-06-22
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -453,13 +453,13 @@
         <v>323</v>
       </c>
       <c r="C2" t="n">
-        <v>440210</v>
+        <v>440134</v>
       </c>
       <c r="D2" t="n">
-        <v>255695</v>
+        <v>251211</v>
       </c>
       <c r="E2" t="n">
-        <v>154996</v>
+        <v>159173</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C3" t="n">
-        <v>23105</v>
+        <v>23052</v>
       </c>
       <c r="D3" t="n">
-        <v>7274</v>
+        <v>6637</v>
       </c>
       <c r="E3" t="n">
-        <v>11429</v>
+        <v>12038</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="C4" t="n">
-        <v>324166</v>
+        <v>325354</v>
       </c>
       <c r="D4" t="n">
-        <v>111542</v>
+        <v>110988</v>
       </c>
       <c r="E4" t="n">
-        <v>137877</v>
+        <v>139251</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="C5" t="n">
-        <v>578114</v>
+        <v>580185</v>
       </c>
       <c r="D5" t="n">
-        <v>207662</v>
+        <v>205076</v>
       </c>
       <c r="E5" t="n">
-        <v>215232</v>
+        <v>219853</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C6" t="n">
         <v>46509</v>
       </c>
       <c r="D6" t="n">
-        <v>22292</v>
+        <v>22042</v>
       </c>
       <c r="E6" t="n">
-        <v>21725</v>
+        <v>21943</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-06-23
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
live order update: 30-day reorder rule + Gigli par (Abby feedback)
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>323</v>
+        <v>63</v>
       </c>
       <c r="C2" t="n">
-        <v>440299</v>
+        <v>60116</v>
       </c>
       <c r="D2" t="n">
-        <v>250812</v>
+        <v>32713</v>
       </c>
       <c r="E2" t="n">
-        <v>160096</v>
+        <v>16582</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>56</v>
+        <v>863</v>
       </c>
       <c r="C3" t="n">
-        <v>23015</v>
+        <v>563676</v>
       </c>
       <c r="D3" t="n">
-        <v>6449</v>
+        <v>205145</v>
       </c>
       <c r="E3" t="n">
-        <v>11981</v>
+        <v>319116</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>649</v>
+        <v>66</v>
       </c>
       <c r="C4" t="n">
-        <v>328279</v>
+        <v>128256</v>
       </c>
       <c r="D4" t="n">
-        <v>111243</v>
+        <v>57221</v>
       </c>
       <c r="E4" t="n">
-        <v>147583</v>
+        <v>32063</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>502</v>
+        <v>123</v>
       </c>
       <c r="C5" t="n">
-        <v>580605</v>
+        <v>336133</v>
       </c>
       <c r="D5" t="n">
-        <v>203552</v>
+        <v>122226</v>
       </c>
       <c r="E5" t="n">
-        <v>223657</v>
+        <v>105713</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>253</v>
+        <v>54</v>
       </c>
       <c r="C6" t="n">
-        <v>46509</v>
+        <v>28495</v>
       </c>
       <c r="D6" t="n">
-        <v>22242</v>
+        <v>14107</v>
       </c>
       <c r="E6" t="n">
-        <v>21730</v>
+        <v>10414</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-06-24
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-06-26
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C2" t="n">
-        <v>60116</v>
+        <v>55076</v>
       </c>
       <c r="D2" t="n">
-        <v>32713</v>
+        <v>31213</v>
       </c>
       <c r="E2" t="n">
-        <v>16582</v>
+        <v>13048</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>863</v>
+        <v>841</v>
       </c>
       <c r="C3" t="n">
-        <v>563676</v>
+        <v>553302</v>
       </c>
       <c r="D3" t="n">
-        <v>205145</v>
+        <v>216176</v>
       </c>
       <c r="E3" t="n">
-        <v>319116</v>
+        <v>296169</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="C4" t="n">
-        <v>128256</v>
+        <v>98623</v>
       </c>
       <c r="D4" t="n">
-        <v>57221</v>
+        <v>47262</v>
       </c>
       <c r="E4" t="n">
-        <v>32063</v>
+        <v>17585</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>123</v>
+        <v>107</v>
       </c>
       <c r="C5" t="n">
-        <v>336133</v>
+        <v>278573</v>
       </c>
       <c r="D5" t="n">
-        <v>122226</v>
+        <v>112754</v>
       </c>
       <c r="E5" t="n">
-        <v>105713</v>
+        <v>65870</v>
       </c>
     </row>
     <row r="6">
@@ -529,13 +529,13 @@
         <v>54</v>
       </c>
       <c r="C6" t="n">
-        <v>28495</v>
+        <v>27587</v>
       </c>
       <c r="D6" t="n">
-        <v>14107</v>
+        <v>13636</v>
       </c>
       <c r="E6" t="n">
-        <v>10414</v>
+        <v>10133</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-06-27
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C2" t="n">
-        <v>53487</v>
+        <v>58209</v>
       </c>
       <c r="D2" t="n">
-        <v>29940</v>
+        <v>33157</v>
       </c>
       <c r="E2" t="n">
-        <v>12541</v>
+        <v>13573</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>830</v>
+        <v>781</v>
       </c>
       <c r="C3" t="n">
-        <v>551802</v>
+        <v>510752</v>
       </c>
       <c r="D3" t="n">
-        <v>220340</v>
+        <v>218349</v>
       </c>
       <c r="E3" t="n">
-        <v>289972</v>
+        <v>250218</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C4" t="n">
-        <v>81466</v>
+        <v>87531</v>
       </c>
       <c r="D4" t="n">
-        <v>40223</v>
+        <v>41312</v>
       </c>
       <c r="E4" t="n">
-        <v>12939</v>
+        <v>16402</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>94</v>
+        <v>112</v>
       </c>
       <c r="C5" t="n">
-        <v>260882</v>
+        <v>292079</v>
       </c>
       <c r="D5" t="n">
-        <v>105106</v>
+        <v>116049</v>
       </c>
       <c r="E5" t="n">
-        <v>57979</v>
+        <v>67828</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C6" t="n">
-        <v>27715</v>
+        <v>27885</v>
       </c>
       <c r="D6" t="n">
-        <v>12942</v>
+        <v>14062</v>
       </c>
       <c r="E6" t="n">
-        <v>10943</v>
+        <v>10000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-06-28
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="C2" t="n">
-        <v>58209</v>
+        <v>65415</v>
       </c>
       <c r="D2" t="n">
-        <v>33157</v>
+        <v>37393</v>
       </c>
       <c r="E2" t="n">
-        <v>13573</v>
+        <v>16058</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>781</v>
+        <v>845</v>
       </c>
       <c r="C3" t="n">
-        <v>510752</v>
+        <v>565462</v>
       </c>
       <c r="D3" t="n">
-        <v>218349</v>
+        <v>232816</v>
       </c>
       <c r="E3" t="n">
-        <v>250218</v>
+        <v>298241</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="C4" t="n">
-        <v>87531</v>
+        <v>92924</v>
       </c>
       <c r="D4" t="n">
-        <v>41312</v>
+        <v>44306</v>
       </c>
       <c r="E4" t="n">
-        <v>16402</v>
+        <v>17830</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>112</v>
+        <v>130</v>
       </c>
       <c r="C5" t="n">
-        <v>292079</v>
+        <v>321298</v>
       </c>
       <c r="D5" t="n">
-        <v>116049</v>
+        <v>123807</v>
       </c>
       <c r="E5" t="n">
-        <v>67828</v>
+        <v>81068</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="C6" t="n">
-        <v>27885</v>
+        <v>31520</v>
       </c>
       <c r="D6" t="n">
-        <v>14062</v>
+        <v>15092</v>
       </c>
       <c r="E6" t="n">
-        <v>10000</v>
+        <v>12732</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-06-29
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="C2" t="n">
-        <v>65415</v>
+        <v>56680</v>
       </c>
       <c r="D2" t="n">
-        <v>37393</v>
+        <v>32525</v>
       </c>
       <c r="E2" t="n">
-        <v>16058</v>
+        <v>12929</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>845</v>
+        <v>789</v>
       </c>
       <c r="C3" t="n">
-        <v>565462</v>
+        <v>522429</v>
       </c>
       <c r="D3" t="n">
-        <v>232816</v>
+        <v>220764</v>
       </c>
       <c r="E3" t="n">
-        <v>298241</v>
+        <v>267398</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C4" t="n">
-        <v>92924</v>
+        <v>92235</v>
       </c>
       <c r="D4" t="n">
-        <v>44306</v>
+        <v>43700</v>
       </c>
       <c r="E4" t="n">
-        <v>17830</v>
+        <v>17648</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C5" t="n">
-        <v>321298</v>
+        <v>316139</v>
       </c>
       <c r="D5" t="n">
-        <v>123807</v>
+        <v>121867</v>
       </c>
       <c r="E5" t="n">
-        <v>81068</v>
+        <v>82405</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C6" t="n">
-        <v>31520</v>
+        <v>29594</v>
       </c>
       <c r="D6" t="n">
-        <v>15092</v>
+        <v>14487</v>
       </c>
       <c r="E6" t="n">
-        <v>12732</v>
+        <v>11199</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-07-01
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-07-02
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-07-03
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C2" t="n">
-        <v>65547</v>
+        <v>63095</v>
       </c>
       <c r="D2" t="n">
-        <v>36454</v>
+        <v>35291</v>
       </c>
       <c r="E2" t="n">
-        <v>17048</v>
+        <v>15550</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>845</v>
+        <v>820</v>
       </c>
       <c r="C3" t="n">
-        <v>578617</v>
+        <v>560300</v>
       </c>
       <c r="D3" t="n">
-        <v>229190</v>
+        <v>230986</v>
       </c>
       <c r="E3" t="n">
-        <v>313592</v>
+        <v>291904</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C4" t="n">
-        <v>67210</v>
+        <v>75718</v>
       </c>
       <c r="D4" t="n">
-        <v>40001</v>
+        <v>46059</v>
       </c>
       <c r="E4" t="n">
-        <v>4245</v>
+        <v>6982</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="C5" t="n">
-        <v>250327</v>
+        <v>273951</v>
       </c>
       <c r="D5" t="n">
-        <v>111308</v>
+        <v>109937</v>
       </c>
       <c r="E5" t="n">
-        <v>61846</v>
+        <v>72743</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C6" t="n">
-        <v>28922</v>
+        <v>31291</v>
       </c>
       <c r="D6" t="n">
-        <v>14060</v>
+        <v>14154</v>
       </c>
       <c r="E6" t="n">
-        <v>11317</v>
+        <v>13577</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-07-04
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="C2" t="n">
-        <v>63095</v>
+        <v>77007</v>
       </c>
       <c r="D2" t="n">
-        <v>35291</v>
+        <v>42591</v>
       </c>
       <c r="E2" t="n">
-        <v>15550</v>
+        <v>20888</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>820</v>
+        <v>929</v>
       </c>
       <c r="C3" t="n">
-        <v>560300</v>
+        <v>663453</v>
       </c>
       <c r="D3" t="n">
-        <v>230986</v>
+        <v>244560</v>
       </c>
       <c r="E3" t="n">
-        <v>291904</v>
+        <v>383397</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C4" t="n">
-        <v>75718</v>
+        <v>85354</v>
       </c>
       <c r="D4" t="n">
-        <v>46059</v>
+        <v>53082</v>
       </c>
       <c r="E4" t="n">
-        <v>6982</v>
+        <v>8319</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>112</v>
+        <v>132</v>
       </c>
       <c r="C5" t="n">
-        <v>273951</v>
+        <v>313947</v>
       </c>
       <c r="D5" t="n">
-        <v>109937</v>
+        <v>117140</v>
       </c>
       <c r="E5" t="n">
-        <v>72743</v>
+        <v>91451</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C6" t="n">
-        <v>31291</v>
+        <v>35231</v>
       </c>
       <c r="D6" t="n">
-        <v>14154</v>
+        <v>14545</v>
       </c>
       <c r="E6" t="n">
-        <v>13577</v>
+        <v>16647</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-07-05
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C2" t="n">
-        <v>77007</v>
+        <v>83226</v>
       </c>
       <c r="D2" t="n">
-        <v>42591</v>
+        <v>45372</v>
       </c>
       <c r="E2" t="n">
-        <v>20888</v>
+        <v>23890</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>929</v>
+        <v>1001</v>
       </c>
       <c r="C3" t="n">
-        <v>663453</v>
+        <v>729668</v>
       </c>
       <c r="D3" t="n">
-        <v>244560</v>
+        <v>244883</v>
       </c>
       <c r="E3" t="n">
-        <v>383397</v>
+        <v>451538</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="C4" t="n">
-        <v>85354</v>
+        <v>87573</v>
       </c>
       <c r="D4" t="n">
-        <v>53082</v>
+        <v>54425</v>
       </c>
       <c r="E4" t="n">
-        <v>8319</v>
+        <v>9198</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="C5" t="n">
-        <v>313947</v>
+        <v>339080</v>
       </c>
       <c r="D5" t="n">
-        <v>117140</v>
+        <v>120176</v>
       </c>
       <c r="E5" t="n">
-        <v>91451</v>
+        <v>106477</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C6" t="n">
-        <v>35231</v>
+        <v>40451</v>
       </c>
       <c r="D6" t="n">
-        <v>14545</v>
+        <v>15982</v>
       </c>
       <c r="E6" t="n">
-        <v>16647</v>
+        <v>20638</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-07-06
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-07-07
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-07-08
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-07-09
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="C2" t="n">
-        <v>76469</v>
+        <v>67672</v>
       </c>
       <c r="D2" t="n">
-        <v>41264</v>
+        <v>40119</v>
       </c>
       <c r="E2" t="n">
-        <v>21255</v>
+        <v>15747</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>932</v>
+        <v>956</v>
       </c>
       <c r="C3" t="n">
-        <v>651679</v>
+        <v>674069</v>
       </c>
       <c r="D3" t="n">
-        <v>237137</v>
+        <v>238332</v>
       </c>
       <c r="E3" t="n">
-        <v>381193</v>
+        <v>403755</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="C4" t="n">
-        <v>91869</v>
+        <v>86615</v>
       </c>
       <c r="D4" t="n">
-        <v>54109</v>
+        <v>52335</v>
       </c>
       <c r="E4" t="n">
-        <v>13357</v>
+        <v>10527</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>143</v>
+        <v>126</v>
       </c>
       <c r="C5" t="n">
-        <v>324720</v>
+        <v>304452</v>
       </c>
       <c r="D5" t="n">
-        <v>118820</v>
+        <v>115888</v>
       </c>
       <c r="E5" t="n">
-        <v>97273</v>
+        <v>78543</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="C6" t="n">
-        <v>33265</v>
+        <v>30771</v>
       </c>
       <c r="D6" t="n">
-        <v>14665</v>
+        <v>13878</v>
       </c>
       <c r="E6" t="n">
-        <v>14514</v>
+        <v>12620</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-07-10
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C2" t="n">
-        <v>67672</v>
+        <v>65766</v>
       </c>
       <c r="D2" t="n">
-        <v>40119</v>
+        <v>38592</v>
       </c>
       <c r="E2" t="n">
-        <v>15747</v>
+        <v>15600</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>956</v>
+        <v>900</v>
       </c>
       <c r="C3" t="n">
-        <v>674069</v>
+        <v>611501</v>
       </c>
       <c r="D3" t="n">
-        <v>238332</v>
+        <v>243877</v>
       </c>
       <c r="E3" t="n">
-        <v>403755</v>
+        <v>333547</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C4" t="n">
-        <v>86615</v>
+        <v>84834</v>
       </c>
       <c r="D4" t="n">
-        <v>52335</v>
+        <v>50178</v>
       </c>
       <c r="E4" t="n">
-        <v>10527</v>
+        <v>10587</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C5" t="n">
-        <v>304452</v>
+        <v>286676</v>
       </c>
       <c r="D5" t="n">
-        <v>115888</v>
+        <v>105098</v>
       </c>
       <c r="E5" t="n">
-        <v>78543</v>
+        <v>70421</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C6" t="n">
-        <v>30771</v>
+        <v>29184</v>
       </c>
       <c r="D6" t="n">
-        <v>13878</v>
+        <v>13766</v>
       </c>
       <c r="E6" t="n">
-        <v>12620</v>
+        <v>11402</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-07-11
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="C2" t="n">
-        <v>65766</v>
+        <v>70490</v>
       </c>
       <c r="D2" t="n">
-        <v>38592</v>
+        <v>40449</v>
       </c>
       <c r="E2" t="n">
-        <v>15600</v>
+        <v>18745</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>900</v>
+        <v>929</v>
       </c>
       <c r="C3" t="n">
-        <v>611501</v>
+        <v>655301</v>
       </c>
       <c r="D3" t="n">
-        <v>243877</v>
+        <v>240109</v>
       </c>
       <c r="E3" t="n">
-        <v>333547</v>
+        <v>381887</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C4" t="n">
-        <v>84834</v>
+        <v>93795</v>
       </c>
       <c r="D4" t="n">
-        <v>50178</v>
+        <v>55350</v>
       </c>
       <c r="E4" t="n">
-        <v>10587</v>
+        <v>14013</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="C5" t="n">
-        <v>286676</v>
+        <v>309854</v>
       </c>
       <c r="D5" t="n">
-        <v>105098</v>
+        <v>110056</v>
       </c>
       <c r="E5" t="n">
-        <v>70421</v>
+        <v>77939</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C6" t="n">
-        <v>29184</v>
+        <v>30395</v>
       </c>
       <c r="D6" t="n">
-        <v>13766</v>
+        <v>13647</v>
       </c>
       <c r="E6" t="n">
-        <v>11402</v>
+        <v>12547</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-07-12
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C2" t="n">
-        <v>70490</v>
+        <v>79392</v>
       </c>
       <c r="D2" t="n">
-        <v>40449</v>
+        <v>45283</v>
       </c>
       <c r="E2" t="n">
-        <v>18745</v>
+        <v>21656</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>929</v>
+        <v>994</v>
       </c>
       <c r="C3" t="n">
-        <v>655301</v>
+        <v>720809</v>
       </c>
       <c r="D3" t="n">
-        <v>240109</v>
+        <v>235491</v>
       </c>
       <c r="E3" t="n">
-        <v>381887</v>
+        <v>453083</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="C4" t="n">
-        <v>93795</v>
+        <v>101726</v>
       </c>
       <c r="D4" t="n">
-        <v>55350</v>
+        <v>58078</v>
       </c>
       <c r="E4" t="n">
-        <v>14013</v>
+        <v>18069</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C5" t="n">
-        <v>309854</v>
+        <v>334946</v>
       </c>
       <c r="D5" t="n">
-        <v>110056</v>
+        <v>114880</v>
       </c>
       <c r="E5" t="n">
-        <v>77939</v>
+        <v>91659</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="C6" t="n">
-        <v>30395</v>
+        <v>34380</v>
       </c>
       <c r="D6" t="n">
-        <v>13647</v>
+        <v>14777</v>
       </c>
       <c r="E6" t="n">
-        <v>12547</v>
+        <v>15251</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-07-13
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="C2" t="n">
-        <v>79392</v>
+        <v>64206</v>
       </c>
       <c r="D2" t="n">
-        <v>45283</v>
+        <v>35010</v>
       </c>
       <c r="E2" t="n">
-        <v>21656</v>
+        <v>17357</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>994</v>
+        <v>961</v>
       </c>
       <c r="C3" t="n">
-        <v>720809</v>
+        <v>685152</v>
       </c>
       <c r="D3" t="n">
-        <v>235491</v>
+        <v>235317</v>
       </c>
       <c r="E3" t="n">
-        <v>453083</v>
+        <v>416823</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C4" t="n">
-        <v>101726</v>
+        <v>103433</v>
       </c>
       <c r="D4" t="n">
-        <v>58078</v>
+        <v>57739</v>
       </c>
       <c r="E4" t="n">
-        <v>18069</v>
+        <v>20813</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C5" t="n">
-        <v>334946</v>
+        <v>334123</v>
       </c>
       <c r="D5" t="n">
-        <v>114880</v>
+        <v>114865</v>
       </c>
       <c r="E5" t="n">
-        <v>91659</v>
+        <v>91781</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C6" t="n">
-        <v>34380</v>
+        <v>32495</v>
       </c>
       <c r="D6" t="n">
-        <v>14777</v>
+        <v>14146</v>
       </c>
       <c r="E6" t="n">
-        <v>15251</v>
+        <v>13964</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-07-14
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C2" t="n">
-        <v>64206</v>
+        <v>64884</v>
       </c>
       <c r="D2" t="n">
-        <v>35010</v>
+        <v>35452</v>
       </c>
       <c r="E2" t="n">
-        <v>17357</v>
+        <v>17658</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>961</v>
+        <v>954</v>
       </c>
       <c r="C3" t="n">
-        <v>685152</v>
+        <v>676545</v>
       </c>
       <c r="D3" t="n">
-        <v>235317</v>
+        <v>236516</v>
       </c>
       <c r="E3" t="n">
-        <v>416823</v>
+        <v>407458</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C4" t="n">
-        <v>103433</v>
+        <v>105960</v>
       </c>
       <c r="D4" t="n">
-        <v>57739</v>
+        <v>59267</v>
       </c>
       <c r="E4" t="n">
-        <v>20813</v>
+        <v>21976</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C5" t="n">
-        <v>334123</v>
+        <v>328684</v>
       </c>
       <c r="D5" t="n">
-        <v>114865</v>
+        <v>112720</v>
       </c>
       <c r="E5" t="n">
-        <v>91781</v>
+        <v>88208</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C6" t="n">
-        <v>32495</v>
+        <v>32522</v>
       </c>
       <c r="D6" t="n">
-        <v>14146</v>
+        <v>15043</v>
       </c>
       <c r="E6" t="n">
-        <v>13964</v>
+        <v>13180</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-07-20
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="C2" t="n">
-        <v>68878</v>
+        <v>71219</v>
       </c>
       <c r="D2" t="n">
-        <v>38594</v>
+        <v>42563</v>
       </c>
       <c r="E2" t="n">
-        <v>18872</v>
+        <v>14794</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>960</v>
+        <v>942</v>
       </c>
       <c r="C3" t="n">
-        <v>683316</v>
+        <v>676356</v>
       </c>
       <c r="D3" t="n">
-        <v>231352</v>
+        <v>237478</v>
       </c>
       <c r="E3" t="n">
-        <v>419928</v>
+        <v>408480</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>62</v>
+        <v>108</v>
       </c>
       <c r="C4" t="n">
-        <v>111964</v>
+        <v>115464</v>
       </c>
       <c r="D4" t="n">
-        <v>59908</v>
+        <v>60108</v>
       </c>
       <c r="E4" t="n">
-        <v>26654</v>
+        <v>76788</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>132</v>
+        <v>206</v>
       </c>
       <c r="C5" t="n">
-        <v>341644</v>
+        <v>345899</v>
       </c>
       <c r="D5" t="n">
-        <v>114816</v>
+        <v>115383</v>
       </c>
       <c r="E5" t="n">
-        <v>97539</v>
+        <v>219990</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="C6" t="n">
-        <v>32278</v>
+        <v>37612</v>
       </c>
       <c r="D6" t="n">
-        <v>14841</v>
+        <v>15647</v>
       </c>
       <c r="E6" t="n">
-        <v>13008</v>
+        <v>17244</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-07-21
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C2" t="n">
-        <v>71219</v>
+        <v>67068</v>
       </c>
       <c r="D2" t="n">
-        <v>42563</v>
+        <v>38530</v>
       </c>
       <c r="E2" t="n">
-        <v>14794</v>
+        <v>14350</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>942</v>
+        <v>925</v>
       </c>
       <c r="C3" t="n">
-        <v>676356</v>
+        <v>667993</v>
       </c>
       <c r="D3" t="n">
-        <v>237478</v>
+        <v>237660</v>
       </c>
       <c r="E3" t="n">
-        <v>408480</v>
+        <v>399401</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C4" t="n">
-        <v>115464</v>
+        <v>118373</v>
       </c>
       <c r="D4" t="n">
-        <v>60108</v>
+        <v>61023</v>
       </c>
       <c r="E4" t="n">
-        <v>76788</v>
+        <v>79252</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C5" t="n">
-        <v>345899</v>
+        <v>335092</v>
       </c>
       <c r="D5" t="n">
-        <v>115383</v>
+        <v>114750</v>
       </c>
       <c r="E5" t="n">
-        <v>219990</v>
+        <v>213857</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C6" t="n">
-        <v>37612</v>
+        <v>36880</v>
       </c>
       <c r="D6" t="n">
-        <v>15647</v>
+        <v>15594</v>
       </c>
       <c r="E6" t="n">
-        <v>17244</v>
+        <v>16683</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-07-22
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -453,10 +453,10 @@
         <v>63</v>
       </c>
       <c r="C2" t="n">
-        <v>69437</v>
+        <v>69154</v>
       </c>
       <c r="D2" t="n">
-        <v>40342</v>
+        <v>39960</v>
       </c>
       <c r="E2" t="n">
         <v>14250</v>
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>905</v>
+        <v>669</v>
       </c>
       <c r="C3" t="n">
-        <v>660622</v>
+        <v>541222</v>
       </c>
       <c r="D3" t="n">
-        <v>230784</v>
+        <v>213259</v>
       </c>
       <c r="E3" t="n">
-        <v>399640</v>
+        <v>304171</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C4" t="n">
-        <v>125270</v>
+        <v>124504</v>
       </c>
       <c r="D4" t="n">
-        <v>63450</v>
+        <v>63045</v>
       </c>
       <c r="E4" t="n">
-        <v>85055</v>
+        <v>84577</v>
       </c>
     </row>
     <row r="5">
@@ -510,13 +510,13 @@
         <v>209</v>
       </c>
       <c r="C5" t="n">
-        <v>350991</v>
+        <v>349272</v>
       </c>
       <c r="D5" t="n">
-        <v>116976</v>
+        <v>116428</v>
       </c>
       <c r="E5" t="n">
-        <v>222931</v>
+        <v>222595</v>
       </c>
     </row>
     <row r="6">
@@ -529,13 +529,13 @@
         <v>75</v>
       </c>
       <c r="C6" t="n">
-        <v>36164</v>
+        <v>34991</v>
       </c>
       <c r="D6" t="n">
-        <v>15267</v>
+        <v>15192</v>
       </c>
       <c r="E6" t="n">
-        <v>16304</v>
+        <v>15308</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-07-23
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="C2" t="n">
-        <v>69154</v>
+        <v>65195</v>
       </c>
       <c r="D2" t="n">
-        <v>39960</v>
+        <v>39528</v>
       </c>
       <c r="E2" t="n">
-        <v>14250</v>
+        <v>11544</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>669</v>
+        <v>677</v>
       </c>
       <c r="C3" t="n">
-        <v>541222</v>
+        <v>556073</v>
       </c>
       <c r="D3" t="n">
-        <v>213259</v>
+        <v>214917</v>
       </c>
       <c r="E3" t="n">
-        <v>304171</v>
+        <v>313140</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="C4" t="n">
-        <v>124504</v>
+        <v>114944</v>
       </c>
       <c r="D4" t="n">
-        <v>63045</v>
+        <v>59332</v>
       </c>
       <c r="E4" t="n">
-        <v>84577</v>
+        <v>79344</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>209</v>
+        <v>190</v>
       </c>
       <c r="C5" t="n">
-        <v>349272</v>
+        <v>315169</v>
       </c>
       <c r="D5" t="n">
-        <v>116428</v>
+        <v>108222</v>
       </c>
       <c r="E5" t="n">
-        <v>222595</v>
+        <v>198296</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C6" t="n">
-        <v>34991</v>
+        <v>33031</v>
       </c>
       <c r="D6" t="n">
-        <v>15192</v>
+        <v>13789</v>
       </c>
       <c r="E6" t="n">
-        <v>15308</v>
+        <v>14828</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-07-24
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C2" t="n">
-        <v>65195</v>
+        <v>58920</v>
       </c>
       <c r="D2" t="n">
-        <v>39528</v>
+        <v>35198</v>
       </c>
       <c r="E2" t="n">
-        <v>11544</v>
+        <v>10084</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>677</v>
+        <v>614</v>
       </c>
       <c r="C3" t="n">
-        <v>556073</v>
+        <v>481517</v>
       </c>
       <c r="D3" t="n">
-        <v>214917</v>
+        <v>215507</v>
       </c>
       <c r="E3" t="n">
-        <v>313140</v>
+        <v>235532</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C4" t="n">
-        <v>114944</v>
+        <v>111253</v>
       </c>
       <c r="D4" t="n">
-        <v>59332</v>
+        <v>58592</v>
       </c>
       <c r="E4" t="n">
-        <v>79344</v>
+        <v>76301</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="C5" t="n">
-        <v>315169</v>
+        <v>303111</v>
       </c>
       <c r="D5" t="n">
-        <v>108222</v>
+        <v>104877</v>
       </c>
       <c r="E5" t="n">
-        <v>198296</v>
+        <v>195294</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="C6" t="n">
-        <v>33031</v>
+        <v>29815</v>
       </c>
       <c r="D6" t="n">
-        <v>13789</v>
+        <v>13284</v>
       </c>
       <c r="E6" t="n">
-        <v>14828</v>
+        <v>12117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-07-25
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="C2" t="n">
-        <v>58920</v>
+        <v>67087</v>
       </c>
       <c r="D2" t="n">
-        <v>35198</v>
+        <v>39652</v>
       </c>
       <c r="E2" t="n">
-        <v>10084</v>
+        <v>12972</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>614</v>
+        <v>689</v>
       </c>
       <c r="C3" t="n">
-        <v>481517</v>
+        <v>544603</v>
       </c>
       <c r="D3" t="n">
-        <v>215507</v>
+        <v>215218</v>
       </c>
       <c r="E3" t="n">
-        <v>235532</v>
+        <v>299010</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C4" t="n">
-        <v>111253</v>
+        <v>122673</v>
       </c>
       <c r="D4" t="n">
-        <v>58592</v>
+        <v>63635</v>
       </c>
       <c r="E4" t="n">
-        <v>76301</v>
+        <v>82240</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="C5" t="n">
-        <v>303111</v>
+        <v>337159</v>
       </c>
       <c r="D5" t="n">
-        <v>104877</v>
+        <v>111050</v>
       </c>
       <c r="E5" t="n">
-        <v>195294</v>
+        <v>211962</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C6" t="n">
-        <v>29815</v>
+        <v>31248</v>
       </c>
       <c r="D6" t="n">
-        <v>13284</v>
+        <v>13894</v>
       </c>
       <c r="E6" t="n">
-        <v>12117</v>
+        <v>13347</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-07-26
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C2" t="n">
-        <v>67087</v>
+        <v>74284</v>
       </c>
       <c r="D2" t="n">
-        <v>39652</v>
+        <v>43379</v>
       </c>
       <c r="E2" t="n">
-        <v>12972</v>
+        <v>15722</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>689</v>
+        <v>732</v>
       </c>
       <c r="C3" t="n">
-        <v>544603</v>
+        <v>599096</v>
       </c>
       <c r="D3" t="n">
-        <v>215218</v>
+        <v>213756</v>
       </c>
       <c r="E3" t="n">
-        <v>299010</v>
+        <v>358422</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="C4" t="n">
-        <v>122673</v>
+        <v>133934</v>
       </c>
       <c r="D4" t="n">
-        <v>63635</v>
+        <v>67325</v>
       </c>
       <c r="E4" t="n">
-        <v>82240</v>
+        <v>89003</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>190</v>
+        <v>204</v>
       </c>
       <c r="C5" t="n">
-        <v>337159</v>
+        <v>364408</v>
       </c>
       <c r="D5" t="n">
-        <v>111050</v>
+        <v>115721</v>
       </c>
       <c r="E5" t="n">
-        <v>211962</v>
+        <v>230668</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C6" t="n">
-        <v>31248</v>
+        <v>33786</v>
       </c>
       <c r="D6" t="n">
-        <v>13894</v>
+        <v>14689</v>
       </c>
       <c r="E6" t="n">
-        <v>13347</v>
+        <v>14810</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-07-27
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-07-28
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C2" t="n">
-        <v>60907</v>
+        <v>62621</v>
       </c>
       <c r="D2" t="n">
-        <v>32772</v>
+        <v>34524</v>
       </c>
       <c r="E2" t="n">
-        <v>13657</v>
+        <v>13495</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>674</v>
+        <v>678</v>
       </c>
       <c r="C3" t="n">
-        <v>527623</v>
+        <v>513948</v>
       </c>
       <c r="D3" t="n">
-        <v>219125</v>
+        <v>216324</v>
       </c>
       <c r="E3" t="n">
-        <v>282269</v>
+        <v>272087</v>
       </c>
     </row>
     <row r="4">
@@ -491,13 +491,13 @@
         <v>113</v>
       </c>
       <c r="C4" t="n">
-        <v>133139</v>
+        <v>138013</v>
       </c>
       <c r="D4" t="n">
-        <v>65884</v>
+        <v>67751</v>
       </c>
       <c r="E4" t="n">
-        <v>91925</v>
+        <v>95545</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="C5" t="n">
-        <v>356172</v>
+        <v>355173</v>
       </c>
       <c r="D5" t="n">
-        <v>113193</v>
+        <v>113308</v>
       </c>
       <c r="E5" t="n">
-        <v>223885</v>
+        <v>221680</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C6" t="n">
-        <v>32351</v>
+        <v>31071</v>
       </c>
       <c r="D6" t="n">
-        <v>13640</v>
+        <v>13004</v>
       </c>
       <c r="E6" t="n">
-        <v>14357</v>
+        <v>13691</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-07-29
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -469,7 +469,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="C3" t="n">
         <v>499037</v>
@@ -478,7 +478,7 @@
         <v>219296</v>
       </c>
       <c r="E3" t="n">
-        <v>253727</v>
+        <v>253605</v>
       </c>
     </row>
     <row r="4">
@@ -488,7 +488,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C4" t="n">
         <v>145932</v>
@@ -497,7 +497,7 @@
         <v>69319</v>
       </c>
       <c r="E4" t="n">
-        <v>102248</v>
+        <v>101937</v>
       </c>
     </row>
     <row r="5">
@@ -507,7 +507,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C5" t="n">
         <v>372122</v>
@@ -516,7 +516,7 @@
         <v>117034</v>
       </c>
       <c r="E5" t="n">
-        <v>233498</v>
+        <v>233594</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
daily order build 2026-07-30
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -450,7 +450,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C2" t="n">
         <v>63859</v>
@@ -459,7 +459,7 @@
         <v>35562</v>
       </c>
       <c r="E2" t="n">
-        <v>13267</v>
+        <v>13106</v>
       </c>
     </row>
     <row r="3">
@@ -469,7 +469,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>626</v>
+        <v>622</v>
       </c>
       <c r="C3" t="n">
         <v>503635</v>
@@ -478,7 +478,7 @@
         <v>221606</v>
       </c>
       <c r="E3" t="n">
-        <v>253206</v>
+        <v>252454</v>
       </c>
     </row>
     <row r="4">
@@ -488,7 +488,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C4" t="n">
         <v>118968</v>
@@ -497,7 +497,7 @@
         <v>59477</v>
       </c>
       <c r="E4" t="n">
-        <v>79422</v>
+        <v>79933</v>
       </c>
     </row>
     <row r="5">
@@ -507,7 +507,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C5" t="n">
         <v>302793</v>
@@ -516,7 +516,7 @@
         <v>112689</v>
       </c>
       <c r="E5" t="n">
-        <v>171672</v>
+        <v>171682</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
daily order build 2026-07-31
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C2" t="n">
-        <v>63859</v>
+        <v>65880</v>
       </c>
       <c r="D2" t="n">
-        <v>35562</v>
+        <v>36520</v>
       </c>
       <c r="E2" t="n">
-        <v>13106</v>
+        <v>13922</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>622</v>
+        <v>640</v>
       </c>
       <c r="C3" t="n">
-        <v>503635</v>
+        <v>525802</v>
       </c>
       <c r="D3" t="n">
-        <v>221606</v>
+        <v>222549</v>
       </c>
       <c r="E3" t="n">
-        <v>252454</v>
+        <v>269882</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>99</v>
+        <v>78</v>
       </c>
       <c r="C4" t="n">
-        <v>118968</v>
+        <v>93338</v>
       </c>
       <c r="D4" t="n">
-        <v>59477</v>
+        <v>47941</v>
       </c>
       <c r="E4" t="n">
-        <v>79933</v>
+        <v>65157</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>171</v>
+        <v>143</v>
       </c>
       <c r="C5" t="n">
-        <v>302793</v>
+        <v>257838</v>
       </c>
       <c r="D5" t="n">
-        <v>112689</v>
+        <v>93580</v>
       </c>
       <c r="E5" t="n">
-        <v>171682</v>
+        <v>140091</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="C6" t="n">
-        <v>29488</v>
+        <v>27534</v>
       </c>
       <c r="D6" t="n">
-        <v>13547</v>
+        <v>12497</v>
       </c>
       <c r="E6" t="n">
-        <v>11666</v>
+        <v>10942</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-08-01
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C2" t="n">
         <v>65880</v>
       </c>
       <c r="D2" t="n">
-        <v>36520</v>
+        <v>35174</v>
       </c>
       <c r="E2" t="n">
-        <v>13922</v>
+        <v>15094</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>640</v>
+        <v>575</v>
       </c>
       <c r="C3" t="n">
-        <v>525802</v>
+        <v>457290</v>
       </c>
       <c r="D3" t="n">
-        <v>222549</v>
+        <v>217184</v>
       </c>
       <c r="E3" t="n">
-        <v>269882</v>
+        <v>440799</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>78</v>
+        <v>120</v>
       </c>
       <c r="C4" t="n">
-        <v>93338</v>
+        <v>99500</v>
       </c>
       <c r="D4" t="n">
-        <v>47941</v>
+        <v>48730</v>
       </c>
       <c r="E4" t="n">
-        <v>65157</v>
+        <v>165826</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>143</v>
+        <v>206</v>
       </c>
       <c r="C5" t="n">
-        <v>257838</v>
+        <v>289360</v>
       </c>
       <c r="D5" t="n">
-        <v>93580</v>
+        <v>100890</v>
       </c>
       <c r="E5" t="n">
-        <v>140091</v>
+        <v>222222</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="C6" t="n">
-        <v>27534</v>
+        <v>27271</v>
       </c>
       <c r="D6" t="n">
-        <v>12497</v>
+        <v>11419</v>
       </c>
       <c r="E6" t="n">
-        <v>10942</v>
+        <v>11770</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-08-02
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C2" t="n">
-        <v>65880</v>
+        <v>71401</v>
       </c>
       <c r="D2" t="n">
-        <v>35174</v>
+        <v>39949</v>
       </c>
       <c r="E2" t="n">
-        <v>15094</v>
+        <v>15813</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>575</v>
+        <v>596</v>
       </c>
       <c r="C3" t="n">
-        <v>457290</v>
+        <v>483599</v>
       </c>
       <c r="D3" t="n">
-        <v>217184</v>
+        <v>216831</v>
       </c>
       <c r="E3" t="n">
-        <v>440799</v>
+        <v>460671</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="C4" t="n">
-        <v>99500</v>
+        <v>102784</v>
       </c>
       <c r="D4" t="n">
-        <v>48730</v>
+        <v>51459</v>
       </c>
       <c r="E4" t="n">
-        <v>165826</v>
+        <v>164677</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>206</v>
+        <v>216</v>
       </c>
       <c r="C5" t="n">
-        <v>289360</v>
+        <v>288682</v>
       </c>
       <c r="D5" t="n">
-        <v>100890</v>
+        <v>97063</v>
       </c>
       <c r="E5" t="n">
-        <v>222222</v>
+        <v>227563</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C6" t="n">
-        <v>27271</v>
+        <v>29351</v>
       </c>
       <c r="D6" t="n">
-        <v>11419</v>
+        <v>12329</v>
       </c>
       <c r="E6" t="n">
-        <v>11770</v>
+        <v>12700</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-08-03
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-08-04
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-08-05
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-08-07
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-08-08
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C2" t="n">
-        <v>70973</v>
+        <v>76871</v>
       </c>
       <c r="D2" t="n">
-        <v>40466</v>
+        <v>43299</v>
       </c>
       <c r="E2" t="n">
-        <v>16072</v>
+        <v>18744</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>496</v>
+        <v>523</v>
       </c>
       <c r="C3" t="n">
-        <v>408635</v>
+        <v>418738</v>
       </c>
       <c r="D3" t="n">
-        <v>207390</v>
+        <v>204006</v>
       </c>
       <c r="E3" t="n">
-        <v>174799</v>
+        <v>188781</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="C4" t="n">
-        <v>103391</v>
+        <v>113304</v>
       </c>
       <c r="D4" t="n">
-        <v>48154</v>
+        <v>50633</v>
       </c>
       <c r="E4" t="n">
-        <v>167353</v>
+        <v>176714</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>202</v>
+        <v>212</v>
       </c>
       <c r="C5" t="n">
-        <v>242508</v>
+        <v>275950</v>
       </c>
       <c r="D5" t="n">
-        <v>82784</v>
+        <v>90747</v>
       </c>
       <c r="E5" t="n">
-        <v>399050</v>
+        <v>434347</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C6" t="n">
-        <v>25614</v>
+        <v>26030</v>
       </c>
       <c r="D6" t="n">
-        <v>12337</v>
+        <v>12581</v>
       </c>
       <c r="E6" t="n">
-        <v>9470</v>
+        <v>9704</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-08-09
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="C2" t="n">
-        <v>76871</v>
+        <v>82764</v>
       </c>
       <c r="D2" t="n">
-        <v>43299</v>
+        <v>46773</v>
       </c>
       <c r="E2" t="n">
-        <v>18744</v>
+        <v>21677</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>523</v>
+        <v>571</v>
       </c>
       <c r="C3" t="n">
-        <v>418738</v>
+        <v>461784</v>
       </c>
       <c r="D3" t="n">
-        <v>204006</v>
+        <v>204354</v>
       </c>
       <c r="E3" t="n">
-        <v>188781</v>
+        <v>231591</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C4" t="n">
-        <v>113304</v>
+        <v>120442</v>
       </c>
       <c r="D4" t="n">
-        <v>50633</v>
+        <v>53040</v>
       </c>
       <c r="E4" t="n">
-        <v>176714</v>
+        <v>182446</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>212</v>
+        <v>225</v>
       </c>
       <c r="C5" t="n">
-        <v>275950</v>
+        <v>302275</v>
       </c>
       <c r="D5" t="n">
-        <v>90747</v>
+        <v>99812</v>
       </c>
       <c r="E5" t="n">
-        <v>434347</v>
+        <v>460583</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="C6" t="n">
-        <v>26030</v>
+        <v>28581</v>
       </c>
       <c r="D6" t="n">
-        <v>12581</v>
+        <v>13225</v>
       </c>
       <c r="E6" t="n">
-        <v>9704</v>
+        <v>11509</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-08-10
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C2" t="n">
-        <v>82764</v>
+        <v>78314</v>
       </c>
       <c r="D2" t="n">
-        <v>46773</v>
+        <v>44934</v>
       </c>
       <c r="E2" t="n">
-        <v>21677</v>
+        <v>19427</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>571</v>
+        <v>527</v>
       </c>
       <c r="C3" t="n">
-        <v>461784</v>
+        <v>426250</v>
       </c>
       <c r="D3" t="n">
-        <v>204354</v>
+        <v>204844</v>
       </c>
       <c r="E3" t="n">
-        <v>231591</v>
+        <v>195804</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C4" t="n">
-        <v>120442</v>
+        <v>120674</v>
       </c>
       <c r="D4" t="n">
-        <v>53040</v>
+        <v>53049</v>
       </c>
       <c r="E4" t="n">
-        <v>182446</v>
+        <v>176555</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="C5" t="n">
-        <v>302275</v>
+        <v>298450</v>
       </c>
       <c r="D5" t="n">
-        <v>99812</v>
+        <v>97989</v>
       </c>
       <c r="E5" t="n">
-        <v>460583</v>
+        <v>443542</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="C6" t="n">
-        <v>28581</v>
+        <v>27582</v>
       </c>
       <c r="D6" t="n">
-        <v>13225</v>
+        <v>13057</v>
       </c>
       <c r="E6" t="n">
-        <v>11509</v>
+        <v>10861</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-08-11
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C2" t="n">
-        <v>78314</v>
+        <v>80169</v>
       </c>
       <c r="D2" t="n">
-        <v>44934</v>
+        <v>46248</v>
       </c>
       <c r="E2" t="n">
-        <v>19427</v>
+        <v>19874</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>527</v>
+        <v>504</v>
       </c>
       <c r="C3" t="n">
-        <v>426250</v>
+        <v>411284</v>
       </c>
       <c r="D3" t="n">
-        <v>204844</v>
+        <v>203691</v>
       </c>
       <c r="E3" t="n">
-        <v>195804</v>
+        <v>182154</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C4" t="n">
-        <v>120674</v>
+        <v>123499</v>
       </c>
       <c r="D4" t="n">
-        <v>53049</v>
+        <v>53419</v>
       </c>
       <c r="E4" t="n">
-        <v>176555</v>
+        <v>174975</v>
       </c>
     </row>
     <row r="5">
@@ -510,13 +510,13 @@
         <v>222</v>
       </c>
       <c r="C5" t="n">
-        <v>298450</v>
+        <v>299235</v>
       </c>
       <c r="D5" t="n">
-        <v>97989</v>
+        <v>99666</v>
       </c>
       <c r="E5" t="n">
-        <v>443542</v>
+        <v>429577</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C6" t="n">
-        <v>27582</v>
+        <v>26343</v>
       </c>
       <c r="D6" t="n">
-        <v>13057</v>
+        <v>12737</v>
       </c>
       <c r="E6" t="n">
-        <v>10861</v>
+        <v>10105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-08-12
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C2" t="n">
-        <v>80169</v>
+        <v>84156</v>
       </c>
       <c r="D2" t="n">
-        <v>46248</v>
+        <v>47678</v>
       </c>
       <c r="E2" t="n">
-        <v>19874</v>
+        <v>22169</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>504</v>
+        <v>495</v>
       </c>
       <c r="C3" t="n">
-        <v>411284</v>
+        <v>408685</v>
       </c>
       <c r="D3" t="n">
-        <v>203691</v>
+        <v>200915</v>
       </c>
       <c r="E3" t="n">
-        <v>182154</v>
+        <v>181813</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C4" t="n">
-        <v>123499</v>
+        <v>129756</v>
       </c>
       <c r="D4" t="n">
-        <v>53419</v>
+        <v>55909</v>
       </c>
       <c r="E4" t="n">
-        <v>174975</v>
+        <v>180763</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="C5" t="n">
-        <v>299235</v>
+        <v>315256</v>
       </c>
       <c r="D5" t="n">
-        <v>99666</v>
+        <v>103391</v>
       </c>
       <c r="E5" t="n">
-        <v>429577</v>
+        <v>441524</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C6" t="n">
-        <v>26343</v>
+        <v>26966</v>
       </c>
       <c r="D6" t="n">
-        <v>12737</v>
+        <v>13296</v>
       </c>
       <c r="E6" t="n">
-        <v>10105</v>
+        <v>10077</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-08-13
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -459,7 +459,7 @@
         <v>46938</v>
       </c>
       <c r="E2" t="n">
-        <v>20432</v>
+        <v>19199</v>
       </c>
     </row>
     <row r="3">
@@ -469,7 +469,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>526</v>
+        <v>534</v>
       </c>
       <c r="C3" t="n">
         <v>429980</v>
@@ -478,7 +478,7 @@
         <v>204210</v>
       </c>
       <c r="E3" t="n">
-        <v>200738</v>
+        <v>202879</v>
       </c>
     </row>
     <row r="4">
@@ -497,7 +497,7 @@
         <v>52530</v>
       </c>
       <c r="E4" t="n">
-        <v>166843</v>
+        <v>167676</v>
       </c>
     </row>
     <row r="5">
@@ -516,7 +516,7 @@
         <v>98398</v>
       </c>
       <c r="E5" t="n">
-        <v>310248</v>
+        <v>311160</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
daily order build 2026-08-14
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C2" t="n">
-        <v>81651</v>
+        <v>81228</v>
       </c>
       <c r="D2" t="n">
-        <v>46938</v>
+        <v>46499</v>
       </c>
       <c r="E2" t="n">
-        <v>19199</v>
+        <v>19518</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>534</v>
+        <v>466</v>
       </c>
       <c r="C3" t="n">
-        <v>429980</v>
+        <v>394491</v>
       </c>
       <c r="D3" t="n">
-        <v>204210</v>
+        <v>198916</v>
       </c>
       <c r="E3" t="n">
-        <v>202879</v>
+        <v>171207</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="C4" t="n">
-        <v>114075</v>
+        <v>103373</v>
       </c>
       <c r="D4" t="n">
-        <v>52530</v>
+        <v>48366</v>
       </c>
       <c r="E4" t="n">
-        <v>167676</v>
+        <v>167843</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="C5" t="n">
-        <v>279728</v>
+        <v>256547</v>
       </c>
       <c r="D5" t="n">
-        <v>98398</v>
+        <v>94975</v>
       </c>
       <c r="E5" t="n">
-        <v>311160</v>
+        <v>296837</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C6" t="n">
-        <v>26214</v>
+        <v>25963</v>
       </c>
       <c r="D6" t="n">
-        <v>13023</v>
+        <v>12764</v>
       </c>
       <c r="E6" t="n">
-        <v>9519</v>
+        <v>9887</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-08-15
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C2" t="n">
-        <v>81228</v>
+        <v>77845</v>
       </c>
       <c r="D2" t="n">
-        <v>46499</v>
+        <v>43447</v>
       </c>
       <c r="E2" t="n">
-        <v>19518</v>
+        <v>18361</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>466</v>
+        <v>484</v>
       </c>
       <c r="C3" t="n">
-        <v>394491</v>
+        <v>394264</v>
       </c>
       <c r="D3" t="n">
-        <v>198916</v>
+        <v>198357</v>
       </c>
       <c r="E3" t="n">
-        <v>171207</v>
+        <v>170607</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C4" t="n">
-        <v>103373</v>
+        <v>115934</v>
       </c>
       <c r="D4" t="n">
-        <v>48366</v>
+        <v>54415</v>
       </c>
       <c r="E4" t="n">
-        <v>167843</v>
+        <v>174700</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>207</v>
+        <v>227</v>
       </c>
       <c r="C5" t="n">
-        <v>256547</v>
+        <v>296977</v>
       </c>
       <c r="D5" t="n">
-        <v>94975</v>
+        <v>106114</v>
       </c>
       <c r="E5" t="n">
-        <v>296837</v>
+        <v>334735</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C6" t="n">
-        <v>25963</v>
+        <v>27209</v>
       </c>
       <c r="D6" t="n">
-        <v>12764</v>
+        <v>12859</v>
       </c>
       <c r="E6" t="n">
-        <v>9887</v>
+        <v>10835</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-08-16
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="C2" t="n">
-        <v>77845</v>
+        <v>82715</v>
       </c>
       <c r="D2" t="n">
-        <v>43447</v>
+        <v>46113</v>
       </c>
       <c r="E2" t="n">
-        <v>18361</v>
+        <v>21211</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>484</v>
+        <v>517</v>
       </c>
       <c r="C3" t="n">
-        <v>394264</v>
+        <v>430759</v>
       </c>
       <c r="D3" t="n">
-        <v>198357</v>
+        <v>206127</v>
       </c>
       <c r="E3" t="n">
-        <v>170607</v>
+        <v>200343</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="C4" t="n">
-        <v>115934</v>
+        <v>123629</v>
       </c>
       <c r="D4" t="n">
-        <v>54415</v>
+        <v>57633</v>
       </c>
       <c r="E4" t="n">
-        <v>174700</v>
+        <v>177458</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>227</v>
+        <v>239</v>
       </c>
       <c r="C5" t="n">
-        <v>296977</v>
+        <v>328218</v>
       </c>
       <c r="D5" t="n">
-        <v>106114</v>
+        <v>112289</v>
       </c>
       <c r="E5" t="n">
-        <v>334735</v>
+        <v>369146</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C6" t="n">
-        <v>27209</v>
+        <v>29140</v>
       </c>
       <c r="D6" t="n">
-        <v>12859</v>
+        <v>13603</v>
       </c>
       <c r="E6" t="n">
-        <v>10835</v>
+        <v>11658</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-08-17
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="C2" t="n">
-        <v>82715</v>
+        <v>79091</v>
       </c>
       <c r="D2" t="n">
-        <v>46113</v>
+        <v>44357</v>
       </c>
       <c r="E2" t="n">
-        <v>21211</v>
+        <v>19535</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>517</v>
+        <v>484</v>
       </c>
       <c r="C3" t="n">
-        <v>430759</v>
+        <v>398329</v>
       </c>
       <c r="D3" t="n">
-        <v>206127</v>
+        <v>204707</v>
       </c>
       <c r="E3" t="n">
-        <v>200343</v>
+        <v>167608</v>
       </c>
     </row>
     <row r="4">
@@ -491,13 +491,13 @@
         <v>124</v>
       </c>
       <c r="C4" t="n">
-        <v>123629</v>
+        <v>125885</v>
       </c>
       <c r="D4" t="n">
-        <v>57633</v>
+        <v>59153</v>
       </c>
       <c r="E4" t="n">
-        <v>177458</v>
+        <v>172794</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>239</v>
+        <v>229</v>
       </c>
       <c r="C5" t="n">
-        <v>328218</v>
+        <v>333236</v>
       </c>
       <c r="D5" t="n">
-        <v>112289</v>
+        <v>109912</v>
       </c>
       <c r="E5" t="n">
-        <v>369146</v>
+        <v>407368</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C6" t="n">
-        <v>29140</v>
+        <v>26558</v>
       </c>
       <c r="D6" t="n">
-        <v>13603</v>
+        <v>13225</v>
       </c>
       <c r="E6" t="n">
-        <v>11658</v>
+        <v>9690</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-08-18
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C2" t="n">
-        <v>79091</v>
+        <v>78883</v>
       </c>
       <c r="D2" t="n">
-        <v>44357</v>
+        <v>44362</v>
       </c>
       <c r="E2" t="n">
-        <v>19535</v>
+        <v>19798</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>484</v>
+        <v>474</v>
       </c>
       <c r="C3" t="n">
-        <v>398329</v>
+        <v>388902</v>
       </c>
       <c r="D3" t="n">
-        <v>204707</v>
+        <v>202162</v>
       </c>
       <c r="E3" t="n">
-        <v>167608</v>
+        <v>160653</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="C4" t="n">
-        <v>125885</v>
+        <v>125463</v>
       </c>
       <c r="D4" t="n">
-        <v>59153</v>
+        <v>58716</v>
       </c>
       <c r="E4" t="n">
-        <v>172794</v>
+        <v>171529</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="C5" t="n">
-        <v>333236</v>
+        <v>328642</v>
       </c>
       <c r="D5" t="n">
-        <v>109912</v>
+        <v>110212</v>
       </c>
       <c r="E5" t="n">
-        <v>407368</v>
+        <v>363518</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C6" t="n">
-        <v>26558</v>
+        <v>25457</v>
       </c>
       <c r="D6" t="n">
-        <v>13225</v>
+        <v>12930</v>
       </c>
       <c r="E6" t="n">
-        <v>9690</v>
+        <v>8807</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-08-19
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -453,13 +453,13 @@
         <v>75</v>
       </c>
       <c r="C2" t="n">
-        <v>78883</v>
+        <v>81459</v>
       </c>
       <c r="D2" t="n">
-        <v>44362</v>
+        <v>45077</v>
       </c>
       <c r="E2" t="n">
-        <v>19798</v>
+        <v>21193</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="C3" t="n">
-        <v>388902</v>
+        <v>391959</v>
       </c>
       <c r="D3" t="n">
-        <v>202162</v>
+        <v>202008</v>
       </c>
       <c r="E3" t="n">
-        <v>160653</v>
+        <v>164551</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C4" t="n">
-        <v>125463</v>
+        <v>132814</v>
       </c>
       <c r="D4" t="n">
-        <v>58716</v>
+        <v>61765</v>
       </c>
       <c r="E4" t="n">
-        <v>171529</v>
+        <v>173964</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>222</v>
+        <v>234</v>
       </c>
       <c r="C5" t="n">
-        <v>328642</v>
+        <v>325517</v>
       </c>
       <c r="D5" t="n">
-        <v>110212</v>
+        <v>111429</v>
       </c>
       <c r="E5" t="n">
-        <v>363518</v>
+        <v>280483</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C6" t="n">
-        <v>25457</v>
+        <v>26475</v>
       </c>
       <c r="D6" t="n">
-        <v>12930</v>
+        <v>14102</v>
       </c>
       <c r="E6" t="n">
-        <v>8807</v>
+        <v>8805</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-08-20
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -478,7 +478,7 @@
         <v>204773</v>
       </c>
       <c r="E3" t="n">
-        <v>183940</v>
+        <v>184259</v>
       </c>
     </row>
     <row r="4">
@@ -488,7 +488,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C4" t="n">
         <v>120142</v>
@@ -497,7 +497,7 @@
         <v>57409</v>
       </c>
       <c r="E4" t="n">
-        <v>170426</v>
+        <v>170503</v>
       </c>
     </row>
     <row r="5">
@@ -507,7 +507,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C5" t="n">
         <v>284894</v>
@@ -516,7 +516,7 @@
         <v>98999</v>
       </c>
       <c r="E5" t="n">
-        <v>277206</v>
+        <v>277913</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
daily order build 2026-08-21
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -453,13 +453,13 @@
         <v>73</v>
       </c>
       <c r="C2" t="n">
-        <v>81563</v>
+        <v>80180</v>
       </c>
       <c r="D2" t="n">
-        <v>45302</v>
+        <v>44012</v>
       </c>
       <c r="E2" t="n">
-        <v>20731</v>
+        <v>20240</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>500</v>
+        <v>457</v>
       </c>
       <c r="C3" t="n">
-        <v>414035</v>
+        <v>350682</v>
       </c>
       <c r="D3" t="n">
-        <v>204773</v>
+        <v>187984</v>
       </c>
       <c r="E3" t="n">
-        <v>184259</v>
+        <v>138790</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="C4" t="n">
-        <v>120142</v>
+        <v>114790</v>
       </c>
       <c r="D4" t="n">
-        <v>57409</v>
+        <v>54884</v>
       </c>
       <c r="E4" t="n">
-        <v>170503</v>
+        <v>171560</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>213</v>
+        <v>198</v>
       </c>
       <c r="C5" t="n">
-        <v>284894</v>
+        <v>274209</v>
       </c>
       <c r="D5" t="n">
-        <v>98999</v>
+        <v>94012</v>
       </c>
       <c r="E5" t="n">
-        <v>277913</v>
+        <v>317377</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C6" t="n">
-        <v>26614</v>
+        <v>25174</v>
       </c>
       <c r="D6" t="n">
-        <v>14562</v>
+        <v>13188</v>
       </c>
       <c r="E6" t="n">
-        <v>8766</v>
+        <v>8659</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-08-22
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="C2" t="n">
-        <v>80180</v>
+        <v>87718</v>
       </c>
       <c r="D2" t="n">
-        <v>44012</v>
+        <v>46736</v>
       </c>
       <c r="E2" t="n">
-        <v>20240</v>
+        <v>25085</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>457</v>
+        <v>477</v>
       </c>
       <c r="C3" t="n">
-        <v>350682</v>
+        <v>375883</v>
       </c>
       <c r="D3" t="n">
-        <v>187984</v>
+        <v>190004</v>
       </c>
       <c r="E3" t="n">
-        <v>138790</v>
+        <v>160948</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="C4" t="n">
-        <v>114790</v>
+        <v>128499</v>
       </c>
       <c r="D4" t="n">
-        <v>54884</v>
+        <v>59632</v>
       </c>
       <c r="E4" t="n">
-        <v>171560</v>
+        <v>183657</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>198</v>
+        <v>215</v>
       </c>
       <c r="C5" t="n">
-        <v>274209</v>
+        <v>320245</v>
       </c>
       <c r="D5" t="n">
-        <v>94012</v>
+        <v>102707</v>
       </c>
       <c r="E5" t="n">
-        <v>317377</v>
+        <v>352025</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C6" t="n">
-        <v>25174</v>
+        <v>23035</v>
       </c>
       <c r="D6" t="n">
-        <v>13188</v>
+        <v>12157</v>
       </c>
       <c r="E6" t="n">
-        <v>8659</v>
+        <v>7439</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-08-23
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C2" t="n">
-        <v>87718</v>
+        <v>93539</v>
       </c>
       <c r="D2" t="n">
-        <v>46736</v>
+        <v>49387</v>
       </c>
       <c r="E2" t="n">
-        <v>25085</v>
+        <v>28734</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>477</v>
+        <v>538</v>
       </c>
       <c r="C3" t="n">
-        <v>375883</v>
+        <v>414215</v>
       </c>
       <c r="D3" t="n">
-        <v>190004</v>
+        <v>198983</v>
       </c>
       <c r="E3" t="n">
-        <v>160948</v>
+        <v>190706</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C4" t="n">
-        <v>128499</v>
+        <v>138225</v>
       </c>
       <c r="D4" t="n">
-        <v>59632</v>
+        <v>62472</v>
       </c>
       <c r="E4" t="n">
-        <v>183657</v>
+        <v>186801</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="C5" t="n">
-        <v>320245</v>
+        <v>355618</v>
       </c>
       <c r="D5" t="n">
-        <v>102707</v>
+        <v>108289</v>
       </c>
       <c r="E5" t="n">
-        <v>352025</v>
+        <v>378931</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C6" t="n">
-        <v>23035</v>
+        <v>24998</v>
       </c>
       <c r="D6" t="n">
-        <v>12157</v>
+        <v>12727</v>
       </c>
       <c r="E6" t="n">
-        <v>7439</v>
+        <v>8800</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-08-24
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="C2" t="n">
-        <v>93539</v>
+        <v>86601</v>
       </c>
       <c r="D2" t="n">
-        <v>49387</v>
+        <v>44534</v>
       </c>
       <c r="E2" t="n">
-        <v>28734</v>
+        <v>26428</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>538</v>
+        <v>501</v>
       </c>
       <c r="C3" t="n">
-        <v>414215</v>
+        <v>389446</v>
       </c>
       <c r="D3" t="n">
-        <v>198983</v>
+        <v>198668</v>
       </c>
       <c r="E3" t="n">
-        <v>190706</v>
+        <v>166126</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C4" t="n">
-        <v>138225</v>
+        <v>137123</v>
       </c>
       <c r="D4" t="n">
-        <v>62472</v>
+        <v>62583</v>
       </c>
       <c r="E4" t="n">
-        <v>186801</v>
+        <v>182476</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="C5" t="n">
-        <v>355618</v>
+        <v>351305</v>
       </c>
       <c r="D5" t="n">
-        <v>108289</v>
+        <v>105748</v>
       </c>
       <c r="E5" t="n">
-        <v>378931</v>
+        <v>369726</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C6" t="n">
-        <v>24998</v>
+        <v>24194</v>
       </c>
       <c r="D6" t="n">
-        <v>12727</v>
+        <v>12663</v>
       </c>
       <c r="E6" t="n">
-        <v>8800</v>
+        <v>8154</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-08-25
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-08-26
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-08-28
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>84</v>
+        <v>67</v>
       </c>
       <c r="C2" t="n">
-        <v>91229</v>
+        <v>83326</v>
       </c>
       <c r="D2" t="n">
-        <v>47904</v>
+        <v>44760</v>
       </c>
       <c r="E2" t="n">
-        <v>32409</v>
+        <v>27093</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>470</v>
+        <v>466</v>
       </c>
       <c r="C3" t="n">
-        <v>385157</v>
+        <v>393947</v>
       </c>
       <c r="D3" t="n">
-        <v>191484</v>
+        <v>199784</v>
       </c>
       <c r="E3" t="n">
-        <v>167152</v>
+        <v>167190</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>147</v>
+        <v>130</v>
       </c>
       <c r="C4" t="n">
-        <v>150337</v>
+        <v>125122</v>
       </c>
       <c r="D4" t="n">
-        <v>67376</v>
+        <v>64082</v>
       </c>
       <c r="E4" t="n">
-        <v>187649</v>
+        <v>149191</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>222</v>
+        <v>205</v>
       </c>
       <c r="C5" t="n">
-        <v>368977</v>
+        <v>333511</v>
       </c>
       <c r="D5" t="n">
-        <v>110159</v>
+        <v>105563</v>
       </c>
       <c r="E5" t="n">
-        <v>373856</v>
+        <v>339121</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C6" t="n">
-        <v>21354</v>
+        <v>21763</v>
       </c>
       <c r="D6" t="n">
-        <v>11946</v>
+        <v>12217</v>
       </c>
       <c r="E6" t="n">
-        <v>6210</v>
+        <v>6263</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-08-29
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -453,13 +453,13 @@
         <v>67</v>
       </c>
       <c r="C2" t="n">
-        <v>83326</v>
+        <v>81305</v>
       </c>
       <c r="D2" t="n">
-        <v>44760</v>
+        <v>44663</v>
       </c>
       <c r="E2" t="n">
-        <v>27093</v>
+        <v>26117</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>466</v>
+        <v>409</v>
       </c>
       <c r="C3" t="n">
-        <v>393947</v>
+        <v>346610</v>
       </c>
       <c r="D3" t="n">
-        <v>199784</v>
+        <v>186375</v>
       </c>
       <c r="E3" t="n">
-        <v>167190</v>
+        <v>132793</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>130</v>
+        <v>108</v>
       </c>
       <c r="C4" t="n">
-        <v>125122</v>
+        <v>105092</v>
       </c>
       <c r="D4" t="n">
-        <v>64082</v>
+        <v>52930</v>
       </c>
       <c r="E4" t="n">
-        <v>149191</v>
+        <v>124215</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>205</v>
+        <v>183</v>
       </c>
       <c r="C5" t="n">
-        <v>333511</v>
+        <v>273756</v>
       </c>
       <c r="D5" t="n">
-        <v>105563</v>
+        <v>103056</v>
       </c>
       <c r="E5" t="n">
-        <v>339121</v>
+        <v>279564</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C6" t="n">
-        <v>21763</v>
+        <v>22288</v>
       </c>
       <c r="D6" t="n">
-        <v>12217</v>
+        <v>12604</v>
       </c>
       <c r="E6" t="n">
-        <v>6263</v>
+        <v>6447</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-08-30
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="C2" t="n">
-        <v>87564</v>
+        <v>93774</v>
       </c>
       <c r="D2" t="n">
-        <v>46692</v>
+        <v>49627</v>
       </c>
       <c r="E2" t="n">
-        <v>29310</v>
+        <v>33850</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>448</v>
+        <v>493</v>
       </c>
       <c r="C3" t="n">
-        <v>380283</v>
+        <v>415590</v>
       </c>
       <c r="D3" t="n">
-        <v>192760</v>
+        <v>194838</v>
       </c>
       <c r="E3" t="n">
-        <v>160720</v>
+        <v>194038</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C4" t="n">
-        <v>118080</v>
+        <v>122392</v>
       </c>
       <c r="D4" t="n">
-        <v>58394</v>
+        <v>60784</v>
       </c>
       <c r="E4" t="n">
-        <v>133733</v>
+        <v>138911</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="C5" t="n">
-        <v>307144</v>
+        <v>303901</v>
       </c>
       <c r="D5" t="n">
-        <v>107998</v>
+        <v>115965</v>
       </c>
       <c r="E5" t="n">
-        <v>312205</v>
+        <v>303964</v>
       </c>
     </row>
     <row r="6">
@@ -529,13 +529,13 @@
         <v>52</v>
       </c>
       <c r="C6" t="n">
-        <v>22415</v>
+        <v>23627</v>
       </c>
       <c r="D6" t="n">
-        <v>12972</v>
+        <v>13754</v>
       </c>
       <c r="E6" t="n">
-        <v>6141</v>
+        <v>6736</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-08-31
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-09-01
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-09-02
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C2" t="n">
-        <v>85967</v>
+        <v>87021</v>
       </c>
       <c r="D2" t="n">
-        <v>43393</v>
+        <v>44832</v>
       </c>
       <c r="E2" t="n">
-        <v>27159</v>
+        <v>26703</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="C3" t="n">
-        <v>378388</v>
+        <v>381270</v>
       </c>
       <c r="D3" t="n">
-        <v>185030</v>
+        <v>180242</v>
       </c>
       <c r="E3" t="n">
-        <v>172822</v>
+        <v>180513</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="C4" t="n">
-        <v>127444</v>
+        <v>130776</v>
       </c>
       <c r="D4" t="n">
-        <v>62053</v>
+        <v>66258</v>
       </c>
       <c r="E4" t="n">
-        <v>116540</v>
+        <v>122854</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C5" t="n">
-        <v>302507</v>
+        <v>318379</v>
       </c>
       <c r="D5" t="n">
-        <v>115612</v>
+        <v>118594</v>
       </c>
       <c r="E5" t="n">
-        <v>226778</v>
+        <v>234853</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C6" t="n">
-        <v>20992</v>
+        <v>22002</v>
       </c>
       <c r="D6" t="n">
-        <v>12764</v>
+        <v>13503</v>
       </c>
       <c r="E6" t="n">
-        <v>5282</v>
+        <v>5518</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-09-03
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C2" t="n">
-        <v>87021</v>
+        <v>84321</v>
       </c>
       <c r="D2" t="n">
-        <v>44832</v>
+        <v>44489</v>
       </c>
       <c r="E2" t="n">
-        <v>26703</v>
+        <v>23854</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="C3" t="n">
-        <v>381270</v>
+        <v>385496</v>
       </c>
       <c r="D3" t="n">
-        <v>180242</v>
+        <v>183161</v>
       </c>
       <c r="E3" t="n">
-        <v>180513</v>
+        <v>177321</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="C4" t="n">
-        <v>130776</v>
+        <v>122891</v>
       </c>
       <c r="D4" t="n">
-        <v>66258</v>
+        <v>63179</v>
       </c>
       <c r="E4" t="n">
-        <v>122854</v>
+        <v>122372</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="C5" t="n">
-        <v>318379</v>
+        <v>290269</v>
       </c>
       <c r="D5" t="n">
-        <v>118594</v>
+        <v>116515</v>
       </c>
       <c r="E5" t="n">
-        <v>234853</v>
+        <v>232514</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C6" t="n">
-        <v>22002</v>
+        <v>22824</v>
       </c>
       <c r="D6" t="n">
-        <v>13503</v>
+        <v>14157</v>
       </c>
       <c r="E6" t="n">
-        <v>5518</v>
+        <v>5716</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-09-04
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C2" t="n">
-        <v>84321</v>
+        <v>84791</v>
       </c>
       <c r="D2" t="n">
-        <v>44489</v>
+        <v>45722</v>
       </c>
       <c r="E2" t="n">
-        <v>23854</v>
+        <v>23634</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>473</v>
+        <v>423</v>
       </c>
       <c r="C3" t="n">
-        <v>385496</v>
+        <v>351815</v>
       </c>
       <c r="D3" t="n">
-        <v>183161</v>
+        <v>169752</v>
       </c>
       <c r="E3" t="n">
-        <v>177321</v>
+        <v>155997</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C4" t="n">
-        <v>122891</v>
+        <v>118604</v>
       </c>
       <c r="D4" t="n">
-        <v>63179</v>
+        <v>61983</v>
       </c>
       <c r="E4" t="n">
-        <v>122372</v>
+        <v>118157</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C5" t="n">
-        <v>290269</v>
+        <v>259274</v>
       </c>
       <c r="D5" t="n">
-        <v>116515</v>
+        <v>92987</v>
       </c>
       <c r="E5" t="n">
-        <v>232514</v>
+        <v>227171</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C6" t="n">
-        <v>22824</v>
+        <v>22424</v>
       </c>
       <c r="D6" t="n">
-        <v>14157</v>
+        <v>13123</v>
       </c>
       <c r="E6" t="n">
-        <v>5716</v>
+        <v>6326</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-09-05
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>74</v>
+        <v>91</v>
       </c>
       <c r="C2" t="n">
-        <v>84791</v>
+        <v>95321</v>
       </c>
       <c r="D2" t="n">
-        <v>45722</v>
+        <v>49860</v>
       </c>
       <c r="E2" t="n">
-        <v>23634</v>
+        <v>30100</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>423</v>
+        <v>458</v>
       </c>
       <c r="C3" t="n">
-        <v>351815</v>
+        <v>386088</v>
       </c>
       <c r="D3" t="n">
-        <v>169752</v>
+        <v>181054</v>
       </c>
       <c r="E3" t="n">
-        <v>155997</v>
+        <v>177639</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="C4" t="n">
-        <v>118604</v>
+        <v>129498</v>
       </c>
       <c r="D4" t="n">
-        <v>61983</v>
+        <v>66333</v>
       </c>
       <c r="E4" t="n">
-        <v>118157</v>
+        <v>125655</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>141</v>
+        <v>152</v>
       </c>
       <c r="C5" t="n">
-        <v>259274</v>
+        <v>283562</v>
       </c>
       <c r="D5" t="n">
-        <v>92987</v>
+        <v>93644</v>
       </c>
       <c r="E5" t="n">
-        <v>227171</v>
+        <v>249368</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C6" t="n">
-        <v>22424</v>
+        <v>23792</v>
       </c>
       <c r="D6" t="n">
-        <v>13123</v>
+        <v>13794</v>
       </c>
       <c r="E6" t="n">
-        <v>6326</v>
+        <v>6905</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-09-06
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="C2" t="n">
-        <v>95321</v>
+        <v>103141</v>
       </c>
       <c r="D2" t="n">
-        <v>49860</v>
+        <v>52962</v>
       </c>
       <c r="E2" t="n">
-        <v>30100</v>
+        <v>34169</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>458</v>
+        <v>488</v>
       </c>
       <c r="C3" t="n">
-        <v>386088</v>
+        <v>429714</v>
       </c>
       <c r="D3" t="n">
-        <v>181054</v>
+        <v>196217</v>
       </c>
       <c r="E3" t="n">
-        <v>177639</v>
+        <v>204982</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C4" t="n">
-        <v>129498</v>
+        <v>137015</v>
       </c>
       <c r="D4" t="n">
-        <v>66333</v>
+        <v>69465</v>
       </c>
       <c r="E4" t="n">
-        <v>125655</v>
+        <v>130506</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>152</v>
+        <v>163</v>
       </c>
       <c r="C5" t="n">
-        <v>283562</v>
+        <v>307370</v>
       </c>
       <c r="D5" t="n">
-        <v>93644</v>
+        <v>101807</v>
       </c>
       <c r="E5" t="n">
-        <v>249368</v>
+        <v>261717</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C6" t="n">
-        <v>23792</v>
+        <v>25486</v>
       </c>
       <c r="D6" t="n">
-        <v>13794</v>
+        <v>14004</v>
       </c>
       <c r="E6" t="n">
-        <v>6905</v>
+        <v>7968</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-09-07
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-09-08
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-09-09
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-09-10
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-09-11
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C2" t="n">
-        <v>98385</v>
+        <v>95798</v>
       </c>
       <c r="D2" t="n">
-        <v>48333</v>
+        <v>45439</v>
       </c>
       <c r="E2" t="n">
-        <v>33427</v>
+        <v>34197</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="C3" t="n">
-        <v>422883</v>
+        <v>426949</v>
       </c>
       <c r="D3" t="n">
-        <v>201077</v>
+        <v>204421</v>
       </c>
       <c r="E3" t="n">
-        <v>195859</v>
+        <v>197737</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="C4" t="n">
-        <v>127878</v>
+        <v>120125</v>
       </c>
       <c r="D4" t="n">
-        <v>61183</v>
+        <v>56706</v>
       </c>
       <c r="E4" t="n">
-        <v>139056</v>
+        <v>135456</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="C5" t="n">
-        <v>271640</v>
+        <v>247839</v>
       </c>
       <c r="D5" t="n">
-        <v>99103</v>
+        <v>90699</v>
       </c>
       <c r="E5" t="n">
-        <v>228965</v>
+        <v>210040</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C6" t="n">
-        <v>27497</v>
+        <v>26083</v>
       </c>
       <c r="D6" t="n">
-        <v>15361</v>
+        <v>14775</v>
       </c>
       <c r="E6" t="n">
-        <v>8353</v>
+        <v>7476</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-09-12
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C2" t="n">
-        <v>95798</v>
+        <v>100122</v>
       </c>
       <c r="D2" t="n">
-        <v>45439</v>
+        <v>48293</v>
       </c>
       <c r="E2" t="n">
-        <v>34197</v>
+        <v>35145</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>502</v>
+        <v>494</v>
       </c>
       <c r="C3" t="n">
-        <v>426949</v>
+        <v>420027</v>
       </c>
       <c r="D3" t="n">
-        <v>204421</v>
+        <v>195551</v>
       </c>
       <c r="E3" t="n">
-        <v>197737</v>
+        <v>198662</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>154</v>
+        <v>170</v>
       </c>
       <c r="C4" t="n">
-        <v>120125</v>
+        <v>136899</v>
       </c>
       <c r="D4" t="n">
-        <v>56706</v>
+        <v>63409</v>
       </c>
       <c r="E4" t="n">
-        <v>135456</v>
+        <v>150421</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>140</v>
+        <v>166</v>
       </c>
       <c r="C5" t="n">
-        <v>247839</v>
+        <v>288085</v>
       </c>
       <c r="D5" t="n">
-        <v>90699</v>
+        <v>101194</v>
       </c>
       <c r="E5" t="n">
-        <v>210040</v>
+        <v>232725</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C6" t="n">
-        <v>26083</v>
+        <v>28114</v>
       </c>
       <c r="D6" t="n">
-        <v>14775</v>
+        <v>15601</v>
       </c>
       <c r="E6" t="n">
-        <v>7476</v>
+        <v>8691</v>
       </c>
     </row>
   </sheetData>

</xml_diff>